<commit_message>
Generacion acta de entrega con excel de audit
</commit_message>
<xml_diff>
--- a/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
+++ b/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto\ControlActivosTI\ControlActivosTI\templates\actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1E8421-4FD4-4039-8E7B-27A22645E2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A692F23-6B3A-4B62-B2D9-9C8BFF29B16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
+    <workbookView xWindow="14290" yWindow="-1820" windowWidth="19420" windowHeight="10300" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$B$1:$I$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$B$1:$I$64</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -996,7 +996,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1119,9 +1119,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1158,9 +1155,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1239,9 +1233,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1263,24 +1254,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1347,9 +1326,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1361,6 +1337,39 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1763,7 +1772,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I63"/>
+  <dimension ref="B1:I64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" style="1" customWidth="1"/>
@@ -1811,9 +1820,9 @@
       <c r="B3" s="27"/>
       <c r="C3" s="28"/>
       <c r="D3" s="41"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="43"/>
+      <c r="E3" s="118"/>
+      <c r="F3" s="118"/>
+      <c r="G3" s="42"/>
       <c r="H3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1825,69 +1834,69 @@
       <c r="B4" s="27"/>
       <c r="C4" s="28"/>
       <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="47" t="s">
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="49">
+      <c r="I4" s="48">
         <v>46097</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="29"/>
       <c r="C5" s="30"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="50"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="49"/>
     </row>
     <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="51" t="s">
+      <c r="B6" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="52"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="75"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
-      <c r="I6" s="77"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="75"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="66" t="s">
+      <c r="B7" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="67"/>
-      <c r="I7" s="68"/>
+      <c r="C7" s="65"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="66"/>
     </row>
     <row r="8" spans="2:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="56"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="119"/>
+      <c r="D8" s="119"/>
+      <c r="E8" s="119"/>
+      <c r="F8" s="119"/>
+      <c r="G8" s="119"/>
+      <c r="H8" s="119"/>
+      <c r="I8" s="54"/>
     </row>
     <row r="9" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="54"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="56"/>
+      <c r="B9" s="53"/>
+      <c r="C9" s="119"/>
+      <c r="D9" s="119"/>
+      <c r="E9" s="119"/>
+      <c r="F9" s="119"/>
+      <c r="G9" s="119"/>
+      <c r="H9" s="119"/>
+      <c r="I9" s="54"/>
     </row>
     <row r="10" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="23" t="s">
@@ -1904,11 +1913,11 @@
       <c r="I10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="80" t="s">
+      <c r="B11" s="78" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="81"/>
-      <c r="D11" s="81"/>
+      <c r="C11" s="79"/>
+      <c r="D11" s="79"/>
       <c r="E11" s="15"/>
       <c r="F11" s="16"/>
       <c r="G11" s="17"/>
@@ -1928,14 +1937,14 @@
       <c r="I12" s="22"/>
     </row>
     <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="70"/>
-      <c r="D13" s="70" t="s">
+      <c r="C13" s="68"/>
+      <c r="D13" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="70"/>
+      <c r="E13" s="68"/>
       <c r="F13" s="10" t="s">
         <v>37</v>
       </c>
@@ -1950,10 +1959,10 @@
       </c>
     </row>
     <row r="14" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="71"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
+      <c r="B14" s="69"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -1970,568 +1979,578 @@
       <c r="I15" s="9"/>
     </row>
     <row r="16" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="78"/>
-      <c r="C16" s="79"/>
-      <c r="D16" s="79"/>
-      <c r="E16" s="79"/>
+      <c r="B16" s="76"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="64"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="65"/>
+      <c r="B17" s="62"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="7"/>
     </row>
     <row r="18" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="86" t="s">
+      <c r="B18" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="87"/>
-      <c r="D18" s="87"/>
-      <c r="E18" s="87"/>
-      <c r="F18" s="87"/>
-      <c r="G18" s="87"/>
-      <c r="H18" s="87"/>
-      <c r="I18" s="88"/>
+      <c r="C18" s="84"/>
+      <c r="D18" s="84"/>
+      <c r="E18" s="84"/>
+      <c r="F18" s="84"/>
+      <c r="G18" s="84"/>
+      <c r="H18" s="84"/>
+      <c r="I18" s="85"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="104" t="s">
+      <c r="B19" s="97" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="105"/>
-      <c r="F19" s="105" t="s">
+      <c r="C19" s="98"/>
+      <c r="D19" s="98"/>
+      <c r="E19" s="98"/>
+      <c r="F19" s="98" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="105"/>
-      <c r="H19" s="105" t="s">
+      <c r="G19" s="98"/>
+      <c r="H19" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="I19" s="106"/>
+      <c r="I19" s="99"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="78" t="s">
+      <c r="B20" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="79"/>
-      <c r="D20" s="79"/>
-      <c r="E20" s="79"/>
-      <c r="F20" s="113"/>
-      <c r="G20" s="113"/>
-      <c r="H20" s="107" t="s">
+      <c r="C20" s="77"/>
+      <c r="D20" s="77"/>
+      <c r="E20" s="77"/>
+      <c r="F20" s="106"/>
+      <c r="G20" s="106"/>
+      <c r="H20" s="100" t="s">
         <v>41</v>
       </c>
-      <c r="I20" s="108"/>
+      <c r="I20" s="101"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="78" t="s">
+      <c r="B21" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="79"/>
-      <c r="D21" s="79"/>
-      <c r="E21" s="79"/>
-      <c r="F21" s="113"/>
-      <c r="G21" s="113"/>
-      <c r="H21" s="109"/>
-      <c r="I21" s="108"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="77"/>
+      <c r="F21" s="106"/>
+      <c r="G21" s="106"/>
+      <c r="H21" s="102"/>
+      <c r="I21" s="101"/>
     </row>
     <row r="22" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="64" t="s">
+      <c r="B22" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="65"/>
-      <c r="D22" s="65"/>
-      <c r="E22" s="65"/>
-      <c r="F22" s="112"/>
-      <c r="G22" s="112"/>
-      <c r="H22" s="110"/>
-      <c r="I22" s="111"/>
+      <c r="C22" s="63"/>
+      <c r="D22" s="63"/>
+      <c r="E22" s="63"/>
+      <c r="F22" s="105"/>
+      <c r="G22" s="105"/>
+      <c r="H22" s="103"/>
+      <c r="I22" s="104"/>
     </row>
     <row r="23" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="72" t="s">
+      <c r="B23" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="73"/>
-      <c r="F23" s="73"/>
-      <c r="G23" s="73"/>
-      <c r="H23" s="73"/>
-      <c r="I23" s="74"/>
+      <c r="C23" s="71"/>
+      <c r="D23" s="71"/>
+      <c r="E23" s="71"/>
+      <c r="F23" s="71"/>
+      <c r="G23" s="71"/>
+      <c r="H23" s="71"/>
+      <c r="I23" s="72"/>
     </row>
     <row r="24" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="53" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="56"/>
+      <c r="C24" s="119"/>
+      <c r="D24" s="119"/>
+      <c r="E24" s="119"/>
+      <c r="F24" s="119"/>
+      <c r="G24" s="119"/>
+      <c r="H24" s="119"/>
+      <c r="I24" s="54"/>
     </row>
     <row r="25" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="54"/>
-      <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="55"/>
-      <c r="G25" s="55"/>
-      <c r="H25" s="55"/>
-      <c r="I25" s="56"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="119"/>
+      <c r="D25" s="119"/>
+      <c r="E25" s="119"/>
+      <c r="F25" s="119"/>
+      <c r="G25" s="119"/>
+      <c r="H25" s="119"/>
+      <c r="I25" s="54"/>
     </row>
     <row r="26" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="55"/>
-      <c r="D26" s="55"/>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="55"/>
-      <c r="H26" s="55"/>
-      <c r="I26" s="56"/>
+      <c r="C26" s="119"/>
+      <c r="D26" s="119"/>
+      <c r="E26" s="119"/>
+      <c r="F26" s="119"/>
+      <c r="G26" s="119"/>
+      <c r="H26" s="119"/>
+      <c r="I26" s="54"/>
     </row>
     <row r="27" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="54" t="s">
+      <c r="B27" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="55"/>
-      <c r="G27" s="55"/>
-      <c r="H27" s="55"/>
-      <c r="I27" s="56"/>
+      <c r="C27" s="119"/>
+      <c r="D27" s="119"/>
+      <c r="E27" s="119"/>
+      <c r="F27" s="119"/>
+      <c r="G27" s="119"/>
+      <c r="H27" s="119"/>
+      <c r="I27" s="54"/>
     </row>
     <row r="28" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="54" t="s">
+      <c r="B28" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="55"/>
-      <c r="H28" s="55"/>
-      <c r="I28" s="56"/>
+      <c r="C28" s="119"/>
+      <c r="D28" s="119"/>
+      <c r="E28" s="119"/>
+      <c r="F28" s="119"/>
+      <c r="G28" s="119"/>
+      <c r="H28" s="119"/>
+      <c r="I28" s="54"/>
     </row>
     <row r="29" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="54" t="s">
+      <c r="B29" s="53" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="56"/>
+      <c r="C29" s="119"/>
+      <c r="D29" s="119"/>
+      <c r="E29" s="119"/>
+      <c r="F29" s="119"/>
+      <c r="G29" s="119"/>
+      <c r="H29" s="119"/>
+      <c r="I29" s="54"/>
     </row>
     <row r="30" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="54" t="s">
+      <c r="B30" s="53" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="56"/>
+      <c r="C30" s="119"/>
+      <c r="D30" s="119"/>
+      <c r="E30" s="119"/>
+      <c r="F30" s="119"/>
+      <c r="G30" s="119"/>
+      <c r="H30" s="119"/>
+      <c r="I30" s="54"/>
     </row>
     <row r="31" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="54" t="s">
+      <c r="B31" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="55"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="55"/>
-      <c r="G31" s="55"/>
-      <c r="H31" s="55"/>
-      <c r="I31" s="56"/>
+      <c r="C31" s="119"/>
+      <c r="D31" s="119"/>
+      <c r="E31" s="119"/>
+      <c r="F31" s="119"/>
+      <c r="G31" s="119"/>
+      <c r="H31" s="119"/>
+      <c r="I31" s="54"/>
     </row>
     <row r="32" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="54" t="s">
+      <c r="B32" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="55"/>
-      <c r="H32" s="55"/>
-      <c r="I32" s="56"/>
+      <c r="C32" s="119"/>
+      <c r="D32" s="119"/>
+      <c r="E32" s="119"/>
+      <c r="F32" s="119"/>
+      <c r="G32" s="119"/>
+      <c r="H32" s="119"/>
+      <c r="I32" s="54"/>
     </row>
     <row r="33" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="54" t="s">
+      <c r="B33" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="56"/>
+      <c r="C33" s="119"/>
+      <c r="D33" s="119"/>
+      <c r="E33" s="119"/>
+      <c r="F33" s="119"/>
+      <c r="G33" s="119"/>
+      <c r="H33" s="119"/>
+      <c r="I33" s="54"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="54" t="s">
+      <c r="B34" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="56"/>
+      <c r="C34" s="119"/>
+      <c r="D34" s="119"/>
+      <c r="E34" s="119"/>
+      <c r="F34" s="119"/>
+      <c r="G34" s="119"/>
+      <c r="H34" s="119"/>
+      <c r="I34" s="54"/>
     </row>
     <row r="35" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="54"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="56"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="119"/>
+      <c r="D35" s="119"/>
+      <c r="E35" s="119"/>
+      <c r="F35" s="119"/>
+      <c r="G35" s="119"/>
+      <c r="H35" s="119"/>
+      <c r="I35" s="54"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="54" t="s">
+      <c r="B36" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="56"/>
+      <c r="C36" s="119"/>
+      <c r="D36" s="119"/>
+      <c r="E36" s="119"/>
+      <c r="F36" s="119"/>
+      <c r="G36" s="119"/>
+      <c r="H36" s="119"/>
+      <c r="I36" s="54"/>
     </row>
     <row r="37" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="57"/>
-      <c r="C37" s="58"/>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58"/>
-      <c r="G37" s="58"/>
-      <c r="H37" s="58"/>
-      <c r="I37" s="59"/>
+      <c r="B37" s="55"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="57"/>
     </row>
     <row r="38" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="58" t="s">
         <v>50</v>
       </c>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="I38" s="62"/>
+      <c r="C38" s="59"/>
+      <c r="D38" s="59"/>
+      <c r="E38" s="59"/>
+      <c r="F38" s="59"/>
+      <c r="G38" s="59"/>
+      <c r="H38" s="59"/>
+      <c r="I38" s="60"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="66" t="s">
+      <c r="B39" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="C39" s="67"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="67"/>
-      <c r="F39" s="67"/>
-      <c r="G39" s="67"/>
-      <c r="H39" s="67"/>
-      <c r="I39" s="68"/>
+      <c r="C39" s="65"/>
+      <c r="D39" s="65"/>
+      <c r="E39" s="65"/>
+      <c r="F39" s="65"/>
+      <c r="G39" s="65"/>
+      <c r="H39" s="65"/>
+      <c r="I39" s="66"/>
     </row>
     <row r="40" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
-      <c r="G40" s="55"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="56"/>
+      <c r="B40" s="53"/>
+      <c r="C40" s="119"/>
+      <c r="D40" s="119"/>
+      <c r="E40" s="119"/>
+      <c r="F40" s="119"/>
+      <c r="G40" s="119"/>
+      <c r="H40" s="119"/>
+      <c r="I40" s="54"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="54" t="s">
+      <c r="B41" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="55"/>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="55"/>
-      <c r="G41" s="55"/>
-      <c r="H41" s="55"/>
-      <c r="I41" s="56"/>
+      <c r="C41" s="119"/>
+      <c r="D41" s="119"/>
+      <c r="E41" s="119"/>
+      <c r="F41" s="119"/>
+      <c r="G41" s="119"/>
+      <c r="H41" s="119"/>
+      <c r="I41" s="54"/>
     </row>
     <row r="42" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="54"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="55"/>
-      <c r="H42" s="55"/>
-      <c r="I42" s="56"/>
+      <c r="B42" s="53"/>
+      <c r="C42" s="119"/>
+      <c r="D42" s="119"/>
+      <c r="E42" s="119"/>
+      <c r="F42" s="119"/>
+      <c r="G42" s="119"/>
+      <c r="H42" s="119"/>
+      <c r="I42" s="54"/>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="54" t="s">
+      <c r="B43" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="C43" s="55"/>
-      <c r="D43" s="55"/>
-      <c r="E43" s="55"/>
-      <c r="F43" s="55"/>
-      <c r="G43" s="55"/>
-      <c r="H43" s="55"/>
-      <c r="I43" s="56"/>
+      <c r="C43" s="119"/>
+      <c r="D43" s="119"/>
+      <c r="E43" s="119"/>
+      <c r="F43" s="119"/>
+      <c r="G43" s="119"/>
+      <c r="H43" s="119"/>
+      <c r="I43" s="54"/>
     </row>
     <row r="44" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="54"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="55"/>
-      <c r="G44" s="55"/>
-      <c r="H44" s="55"/>
-      <c r="I44" s="56"/>
+      <c r="B44" s="53"/>
+      <c r="C44" s="119"/>
+      <c r="D44" s="119"/>
+      <c r="E44" s="119"/>
+      <c r="F44" s="119"/>
+      <c r="G44" s="119"/>
+      <c r="H44" s="119"/>
+      <c r="I44" s="54"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="54" t="s">
+      <c r="B45" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="C45" s="55"/>
-      <c r="D45" s="55"/>
-      <c r="E45" s="55"/>
-      <c r="F45" s="55"/>
-      <c r="G45" s="55"/>
-      <c r="H45" s="55"/>
-      <c r="I45" s="56"/>
+      <c r="C45" s="119"/>
+      <c r="D45" s="119"/>
+      <c r="E45" s="119"/>
+      <c r="F45" s="119"/>
+      <c r="G45" s="119"/>
+      <c r="H45" s="119"/>
+      <c r="I45" s="54"/>
     </row>
     <row r="46" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="54"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="55"/>
-      <c r="F46" s="55"/>
-      <c r="G46" s="55"/>
-      <c r="H46" s="55"/>
-      <c r="I46" s="56"/>
+      <c r="B46" s="53"/>
+      <c r="C46" s="119"/>
+      <c r="D46" s="119"/>
+      <c r="E46" s="119"/>
+      <c r="F46" s="119"/>
+      <c r="G46" s="119"/>
+      <c r="H46" s="119"/>
+      <c r="I46" s="54"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="54" t="s">
+      <c r="B47" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C47" s="55"/>
-      <c r="D47" s="55"/>
-      <c r="E47" s="55"/>
-      <c r="F47" s="55"/>
-      <c r="G47" s="55"/>
-      <c r="H47" s="55"/>
-      <c r="I47" s="56"/>
+      <c r="C47" s="119"/>
+      <c r="D47" s="119"/>
+      <c r="E47" s="119"/>
+      <c r="F47" s="119"/>
+      <c r="G47" s="119"/>
+      <c r="H47" s="119"/>
+      <c r="I47" s="54"/>
     </row>
     <row r="48" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="54"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="56"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="119"/>
+      <c r="D48" s="119"/>
+      <c r="E48" s="119"/>
+      <c r="F48" s="119"/>
+      <c r="G48" s="119"/>
+      <c r="H48" s="119"/>
+      <c r="I48" s="54"/>
     </row>
     <row r="49" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="54" t="s">
+      <c r="B49" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="56"/>
+      <c r="C49" s="119"/>
+      <c r="D49" s="119"/>
+      <c r="E49" s="119"/>
+      <c r="F49" s="119"/>
+      <c r="G49" s="119"/>
+      <c r="H49" s="119"/>
+      <c r="I49" s="54"/>
     </row>
     <row r="50" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="54" t="s">
+      <c r="B50" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="55"/>
-      <c r="F50" s="55"/>
-      <c r="G50" s="55"/>
-      <c r="H50" s="55"/>
-      <c r="I50" s="56"/>
-    </row>
-    <row r="51" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="89" t="s">
+      <c r="C50" s="119"/>
+      <c r="D50" s="119"/>
+      <c r="E50" s="119"/>
+      <c r="F50" s="119"/>
+      <c r="G50" s="119"/>
+      <c r="H50" s="119"/>
+      <c r="I50" s="54"/>
+    </row>
+    <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="86" t="s">
         <v>31</v>
       </c>
-      <c r="C51" s="90"/>
-      <c r="D51" s="90"/>
-      <c r="E51" s="90"/>
-      <c r="F51" s="90"/>
-      <c r="G51" s="90"/>
-      <c r="H51" s="90"/>
-      <c r="I51" s="91"/>
-    </row>
-    <row r="52" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="86" t="s">
+      <c r="C51" s="120"/>
+      <c r="D51" s="120"/>
+      <c r="E51" s="120"/>
+      <c r="F51" s="120"/>
+      <c r="G51" s="120"/>
+      <c r="H51" s="120"/>
+      <c r="I51" s="87"/>
+    </row>
+    <row r="52" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="115"/>
+      <c r="C52" s="116"/>
+      <c r="D52" s="116"/>
+      <c r="E52" s="116"/>
+      <c r="F52" s="116"/>
+      <c r="G52" s="116"/>
+      <c r="H52" s="116"/>
+      <c r="I52" s="117"/>
+    </row>
+    <row r="53" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="C52" s="87"/>
-      <c r="D52" s="87"/>
-      <c r="E52" s="87"/>
-      <c r="F52" s="87"/>
-      <c r="G52" s="87"/>
-      <c r="H52" s="87"/>
-      <c r="I52" s="88"/>
-    </row>
-    <row r="53" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="114"/>
-      <c r="C53" s="115"/>
-      <c r="D53" s="115"/>
-      <c r="E53" s="115"/>
-      <c r="F53" s="115"/>
-      <c r="G53" s="115"/>
-      <c r="H53" s="115"/>
-      <c r="I53" s="116"/>
+      <c r="C53" s="84"/>
+      <c r="D53" s="84"/>
+      <c r="E53" s="84"/>
+      <c r="F53" s="84"/>
+      <c r="G53" s="84"/>
+      <c r="H53" s="84"/>
+      <c r="I53" s="85"/>
     </row>
     <row r="54" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="117"/>
-      <c r="C54" s="118"/>
-      <c r="D54" s="118"/>
-      <c r="E54" s="118"/>
-      <c r="F54" s="118"/>
-      <c r="G54" s="118"/>
-      <c r="H54" s="118"/>
-      <c r="I54" s="119"/>
-    </row>
-    <row r="55" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="120"/>
+      <c r="B54" s="107"/>
+      <c r="C54" s="108"/>
+      <c r="D54" s="108"/>
+      <c r="E54" s="108"/>
+      <c r="F54" s="108"/>
+      <c r="G54" s="108"/>
+      <c r="H54" s="108"/>
+      <c r="I54" s="109"/>
+    </row>
+    <row r="55" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="110"/>
       <c r="C55" s="121"/>
       <c r="D55" s="121"/>
       <c r="E55" s="121"/>
       <c r="F55" s="121"/>
       <c r="G55" s="121"/>
       <c r="H55" s="121"/>
-      <c r="I55" s="122"/>
-    </row>
-    <row r="56" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="83" t="s">
+      <c r="I55" s="111"/>
+    </row>
+    <row r="56" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="112"/>
+      <c r="C56" s="113"/>
+      <c r="D56" s="113"/>
+      <c r="E56" s="113"/>
+      <c r="F56" s="113"/>
+      <c r="G56" s="113"/>
+      <c r="H56" s="113"/>
+      <c r="I56" s="114"/>
+    </row>
+    <row r="57" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="80" t="s">
         <v>53</v>
       </c>
-      <c r="C56" s="84"/>
-      <c r="D56" s="84"/>
-      <c r="E56" s="84"/>
-      <c r="F56" s="84"/>
-      <c r="G56" s="84"/>
-      <c r="H56" s="84"/>
-      <c r="I56" s="85"/>
-    </row>
-    <row r="57" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="93" t="s">
+      <c r="C57" s="81"/>
+      <c r="D57" s="81"/>
+      <c r="E57" s="81"/>
+      <c r="F57" s="81"/>
+      <c r="G57" s="81"/>
+      <c r="H57" s="81"/>
+      <c r="I57" s="82"/>
+    </row>
+    <row r="58" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="C57" s="94"/>
-      <c r="D57" s="92" t="s">
+      <c r="C58" s="122"/>
+      <c r="D58" s="123" t="s">
         <v>16</v>
       </c>
-      <c r="E57" s="92"/>
-      <c r="F57" s="92"/>
-      <c r="G57" s="95" t="s">
+      <c r="E58" s="123"/>
+      <c r="F58" s="123"/>
+      <c r="G58" s="124" t="s">
         <v>15</v>
       </c>
-      <c r="H57" s="82"/>
-      <c r="I57" s="28"/>
-    </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B58" s="93" t="s">
+      <c r="H58" s="125"/>
+      <c r="I58" s="28"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B59" s="88" t="s">
         <v>14</v>
       </c>
-      <c r="C58" s="94"/>
-      <c r="D58" s="92" t="s">
+      <c r="C59" s="122"/>
+      <c r="D59" s="123" t="s">
         <v>17</v>
       </c>
-      <c r="E58" s="92"/>
-      <c r="F58" s="92"/>
-      <c r="G58" s="95"/>
-      <c r="H58" s="82"/>
-      <c r="I58" s="28"/>
-    </row>
-    <row r="59" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="93"/>
-      <c r="C59" s="94"/>
-      <c r="D59" s="92"/>
-      <c r="E59" s="92"/>
-      <c r="F59" s="92"/>
-      <c r="G59" s="95"/>
-      <c r="H59" s="82"/>
+      <c r="E59" s="123"/>
+      <c r="F59" s="123"/>
+      <c r="G59" s="124"/>
+      <c r="H59" s="125"/>
       <c r="I59" s="28"/>
     </row>
-    <row r="60" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="96" t="s">
+    <row r="60" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="88"/>
+      <c r="C60" s="122"/>
+      <c r="D60" s="123"/>
+      <c r="E60" s="123"/>
+      <c r="F60" s="123"/>
+      <c r="G60" s="124"/>
+      <c r="H60" s="125"/>
+      <c r="I60" s="28"/>
+    </row>
+    <row r="61" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="89" t="s">
         <v>54</v>
       </c>
-      <c r="C60" s="97"/>
-      <c r="D60" s="97"/>
-      <c r="E60" s="97"/>
-      <c r="F60" s="97"/>
-      <c r="G60" s="97"/>
-      <c r="H60" s="97"/>
-      <c r="I60" s="98"/>
-    </row>
-    <row r="61" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="93" t="s">
+      <c r="C61" s="90"/>
+      <c r="D61" s="90"/>
+      <c r="E61" s="90"/>
+      <c r="F61" s="90"/>
+      <c r="G61" s="90"/>
+      <c r="H61" s="90"/>
+      <c r="I61" s="91"/>
+    </row>
+    <row r="62" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="C61" s="94"/>
-      <c r="D61" s="92"/>
-      <c r="E61" s="92"/>
-      <c r="F61" s="92"/>
-      <c r="G61" s="95" t="s">
+      <c r="C62" s="122"/>
+      <c r="D62" s="123"/>
+      <c r="E62" s="123"/>
+      <c r="F62" s="123"/>
+      <c r="G62" s="124" t="s">
         <v>15</v>
       </c>
-      <c r="H61" s="82"/>
-      <c r="I61" s="28"/>
-    </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B62" s="93" t="s">
+      <c r="H62" s="125"/>
+      <c r="I62" s="28"/>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B63" s="88" t="s">
         <v>14</v>
       </c>
-      <c r="C62" s="94"/>
-      <c r="D62" s="92"/>
-      <c r="E62" s="92"/>
-      <c r="F62" s="92"/>
-      <c r="G62" s="95"/>
-      <c r="H62" s="82"/>
-      <c r="I62" s="28"/>
-    </row>
-    <row r="63" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="101"/>
-      <c r="C63" s="102"/>
-      <c r="D63" s="103"/>
-      <c r="E63" s="103"/>
-      <c r="F63" s="103"/>
-      <c r="G63" s="99"/>
-      <c r="H63" s="100"/>
-      <c r="I63" s="30"/>
+      <c r="C63" s="122"/>
+      <c r="D63" s="123"/>
+      <c r="E63" s="123"/>
+      <c r="F63" s="123"/>
+      <c r="G63" s="124"/>
+      <c r="H63" s="125"/>
+      <c r="I63" s="28"/>
+    </row>
+    <row r="64" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="94"/>
+      <c r="C64" s="95"/>
+      <c r="D64" s="96"/>
+      <c r="E64" s="96"/>
+      <c r="F64" s="96"/>
+      <c r="G64" s="92"/>
+      <c r="H64" s="93"/>
+      <c r="I64" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="75">
-    <mergeCell ref="B53:I55"/>
+  <mergeCells count="76">
+    <mergeCell ref="B54:I56"/>
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="B50:I50"/>
     <mergeCell ref="B32:I32"/>
@@ -2541,6 +2560,7 @@
     <mergeCell ref="B43:I44"/>
     <mergeCell ref="B45:I46"/>
     <mergeCell ref="B47:I48"/>
+    <mergeCell ref="B52:I52"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="F19:G19"/>
@@ -2552,24 +2572,24 @@
     <mergeCell ref="F21:G21"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B60:I60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="G61:G63"/>
-    <mergeCell ref="H61:I63"/>
-    <mergeCell ref="B62:C63"/>
-    <mergeCell ref="D62:F63"/>
-    <mergeCell ref="H57:I59"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="G62:G64"/>
+    <mergeCell ref="H62:I64"/>
+    <mergeCell ref="B63:C64"/>
+    <mergeCell ref="D63:F64"/>
+    <mergeCell ref="H58:I60"/>
+    <mergeCell ref="B57:I57"/>
+    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B24:I25"/>
     <mergeCell ref="B34:I35"/>
     <mergeCell ref="B51:I51"/>
-    <mergeCell ref="D57:F57"/>
-    <mergeCell ref="B58:C59"/>
-    <mergeCell ref="D58:F59"/>
-    <mergeCell ref="G57:G59"/>
-    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="D58:F58"/>
+    <mergeCell ref="B59:C60"/>
+    <mergeCell ref="D59:F60"/>
+    <mergeCell ref="G58:G60"/>
+    <mergeCell ref="B58:C58"/>
     <mergeCell ref="B27:I27"/>
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B29:I29"/>
@@ -2611,7 +2631,7 @@
   <pageMargins left="0.62992125984251968" right="0.23622047244094491" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="58" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="51" max="16383" man="1"/>
+    <brk id="52" min="1" max="8" man="1"/>
   </rowBreaks>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="1" max="1048575" man="1"/>

</xml_diff>